<commit_message>
added choosable split for some events
</commit_message>
<xml_diff>
--- a/EventsEtnaCLASS_Final.xlsx
+++ b/EventsEtnaCLASS_Final.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Archivio_Lorenzo\DOTTORATO\Progetti\TESI_Code_Rev\Tesi_Code_Revision\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Archivio_Lorenzo\DOTTORATO\Dottorato\Progetti\Unet3D_gatedConv3D_Model_PacketProj-20260324T101554Z-1-001\cleaned-repo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0A68EC0-6B9E-4A19-AD3E-E6E0377A7D16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2178B41-3B92-4434-A0B2-24E0D6571ACE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="13">
   <si>
     <t>Date</t>
   </si>
@@ -66,6 +66,12 @@
   </si>
   <si>
     <t>n.o eruptions per class</t>
+  </si>
+  <si>
+    <t>Split</t>
+  </si>
+  <si>
+    <t>train</t>
   </si>
 </sst>
 </file>
@@ -145,7 +151,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -183,11 +189,65 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -231,9 +291,6 @@
     <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -243,9 +300,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normale" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="5">
     <dxf>
@@ -357,12 +427,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B5B07F33-BEC8-439A-A8B4-3C3D16100EC6}" name="Tabella1" displayName="Tabella1" ref="H1:J5" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B5B07F33-BEC8-439A-A8B4-3C3D16100EC6}" name="Tabella1" displayName="Tabella1" ref="H1:J5" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
   <autoFilter ref="H1:J5" xr:uid="{B5B07F33-BEC8-439A-A8B4-3C3D16100EC6}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{ACC8CF46-AA7A-4965-BF58-45276E8031BD}" name="Class" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{AD3397D4-1C4A-48CA-AEBF-5647EC83F975}" name="Meaning" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{B4CEE906-0859-4F25-8673-397F88A3D8E2}" name="n.o eruptions per class" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{ACC8CF46-AA7A-4965-BF58-45276E8031BD}" name="Class" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{AD3397D4-1C4A-48CA-AEBF-5647EC83F975}" name="Meaning" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{B4CEE906-0859-4F25-8673-397F88A3D8E2}" name="n.o eruptions per class" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -596,6 +666,9 @@
       <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
+      <c r="F1" s="23" t="s">
+        <v>11</v>
+      </c>
       <c r="H1" s="4" t="s">
         <v>4</v>
       </c>
@@ -617,16 +690,17 @@
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
       <c r="D2" s="14"/>
-      <c r="E2" s="17">
+      <c r="E2" s="20">
         <v>3</v>
       </c>
+      <c r="F2" s="24"/>
       <c r="H2" s="4">
         <v>1</v>
       </c>
       <c r="I2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="J2" s="20">
+      <c r="J2" s="19">
         <v>34</v>
       </c>
     </row>
@@ -637,9 +711,10 @@
       <c r="B3" s="12"/>
       <c r="C3" s="12"/>
       <c r="D3" s="14"/>
-      <c r="E3" s="7">
+      <c r="E3" s="21">
         <v>1</v>
       </c>
+      <c r="F3" s="24"/>
       <c r="H3" s="4">
         <v>2</v>
       </c>
@@ -657,9 +732,10 @@
       <c r="B4" s="12"/>
       <c r="C4" s="12"/>
       <c r="D4" s="14"/>
-      <c r="E4" s="7">
+      <c r="E4" s="21">
         <v>1</v>
       </c>
+      <c r="F4" s="24"/>
       <c r="H4" s="4">
         <v>3</v>
       </c>
@@ -677,9 +753,10 @@
       <c r="B5" s="12"/>
       <c r="C5" s="12"/>
       <c r="D5" s="14"/>
-      <c r="E5" s="7">
+      <c r="E5" s="21">
         <v>1</v>
       </c>
+      <c r="F5" s="24"/>
       <c r="H5" s="4">
         <v>4</v>
       </c>
@@ -697,9 +774,10 @@
       <c r="B6" s="12"/>
       <c r="C6" s="12"/>
       <c r="D6" s="14"/>
-      <c r="E6" s="7">
+      <c r="E6" s="21">
         <v>3</v>
       </c>
+      <c r="F6" s="24"/>
     </row>
     <row r="7" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
@@ -708,9 +786,10 @@
       <c r="B7" s="12"/>
       <c r="C7" s="12"/>
       <c r="D7" s="14"/>
-      <c r="E7" s="7">
+      <c r="E7" s="21">
         <v>1</v>
       </c>
+      <c r="F7" s="24"/>
     </row>
     <row r="8" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
@@ -719,9 +798,10 @@
       <c r="B8" s="12"/>
       <c r="C8" s="12"/>
       <c r="D8" s="14"/>
-      <c r="E8" s="7">
+      <c r="E8" s="21">
         <v>1</v>
       </c>
+      <c r="F8" s="24"/>
     </row>
     <row r="9" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
@@ -730,9 +810,10 @@
       <c r="B9" s="12"/>
       <c r="C9" s="12"/>
       <c r="D9" s="14"/>
-      <c r="E9" s="7">
+      <c r="E9" s="21">
         <v>1</v>
       </c>
+      <c r="F9" s="24"/>
     </row>
     <row r="10" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5">
@@ -741,9 +822,10 @@
       <c r="B10" s="12"/>
       <c r="C10" s="12"/>
       <c r="D10" s="14"/>
-      <c r="E10" s="7">
+      <c r="E10" s="21">
         <v>1</v>
       </c>
+      <c r="F10" s="24"/>
     </row>
     <row r="11" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
@@ -752,9 +834,10 @@
       <c r="B11" s="12"/>
       <c r="C11" s="12"/>
       <c r="D11" s="14"/>
-      <c r="E11" s="7">
+      <c r="E11" s="21">
         <v>1</v>
       </c>
+      <c r="F11" s="24"/>
     </row>
     <row r="12" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5">
@@ -763,9 +846,10 @@
       <c r="B12" s="12"/>
       <c r="C12" s="12"/>
       <c r="D12" s="14"/>
-      <c r="E12" s="7">
+      <c r="E12" s="21">
         <v>1</v>
       </c>
+      <c r="F12" s="24"/>
     </row>
     <row r="13" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5">
@@ -774,9 +858,10 @@
       <c r="B13" s="12"/>
       <c r="C13" s="12"/>
       <c r="D13" s="14"/>
-      <c r="E13" s="7">
+      <c r="E13" s="21">
         <v>1</v>
       </c>
+      <c r="F13" s="24"/>
     </row>
     <row r="14" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5">
@@ -785,9 +870,10 @@
       <c r="B14" s="12"/>
       <c r="C14" s="12"/>
       <c r="D14" s="14"/>
-      <c r="E14" s="7">
+      <c r="E14" s="21">
         <v>4</v>
       </c>
+      <c r="F14" s="24"/>
     </row>
     <row r="15" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="5">
@@ -796,9 +882,10 @@
       <c r="B15" s="12"/>
       <c r="C15" s="12"/>
       <c r="D15" s="14"/>
-      <c r="E15" s="7">
+      <c r="E15" s="21">
         <v>1</v>
       </c>
+      <c r="F15" s="24"/>
     </row>
     <row r="16" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="5">
@@ -807,9 +894,10 @@
       <c r="B16" s="12"/>
       <c r="C16" s="12"/>
       <c r="D16" s="14"/>
-      <c r="E16" s="7">
+      <c r="E16" s="21">
         <v>3</v>
       </c>
+      <c r="F16" s="24"/>
     </row>
     <row r="17" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="5">
@@ -818,9 +906,10 @@
       <c r="B17" s="12"/>
       <c r="C17" s="12"/>
       <c r="D17" s="14"/>
-      <c r="E17" s="7">
+      <c r="E17" s="21">
         <v>3</v>
       </c>
+      <c r="F17" s="24"/>
     </row>
     <row r="18" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="5">
@@ -829,9 +918,10 @@
       <c r="B18" s="12"/>
       <c r="C18" s="12"/>
       <c r="D18" s="14"/>
-      <c r="E18" s="7">
+      <c r="E18" s="21">
         <v>3</v>
       </c>
+      <c r="F18" s="24"/>
     </row>
     <row r="19" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="5">
@@ -840,9 +930,10 @@
       <c r="B19" s="12"/>
       <c r="C19" s="12"/>
       <c r="D19" s="14"/>
-      <c r="E19" s="7">
+      <c r="E19" s="21">
         <v>2</v>
       </c>
+      <c r="F19" s="24"/>
     </row>
     <row r="20" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="5">
@@ -851,9 +942,10 @@
       <c r="B20" s="12"/>
       <c r="C20" s="12"/>
       <c r="D20" s="14"/>
-      <c r="E20" s="7">
+      <c r="E20" s="21">
         <v>2</v>
       </c>
+      <c r="F20" s="24"/>
     </row>
     <row r="21" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="5">
@@ -862,9 +954,10 @@
       <c r="B21" s="12"/>
       <c r="C21" s="12"/>
       <c r="D21" s="14"/>
-      <c r="E21" s="7">
+      <c r="E21" s="21">
         <v>3</v>
       </c>
+      <c r="F21" s="24"/>
     </row>
     <row r="22" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="5">
@@ -873,9 +966,10 @@
       <c r="B22" s="12"/>
       <c r="C22" s="12"/>
       <c r="D22" s="14"/>
-      <c r="E22" s="7">
+      <c r="E22" s="21">
         <v>2</v>
       </c>
+      <c r="F22" s="24"/>
     </row>
     <row r="23" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="5">
@@ -884,9 +978,10 @@
       <c r="B23" s="12"/>
       <c r="C23" s="12"/>
       <c r="D23" s="14"/>
-      <c r="E23" s="7">
+      <c r="E23" s="21">
         <v>1</v>
       </c>
+      <c r="F23" s="24"/>
       <c r="I23" s="11"/>
     </row>
     <row r="24" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -896,9 +991,10 @@
       <c r="B24" s="12"/>
       <c r="C24" s="12"/>
       <c r="D24" s="7"/>
-      <c r="E24" s="7">
+      <c r="E24" s="21">
         <v>3</v>
       </c>
+      <c r="F24" s="24"/>
     </row>
     <row r="25" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="5">
@@ -907,9 +1003,10 @@
       <c r="B25" s="12"/>
       <c r="C25" s="12"/>
       <c r="D25" s="7"/>
-      <c r="E25" s="7">
+      <c r="E25" s="21">
         <v>3</v>
       </c>
+      <c r="F25" s="24"/>
     </row>
     <row r="26" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="5">
@@ -918,9 +1015,10 @@
       <c r="B26" s="12"/>
       <c r="C26" s="12"/>
       <c r="D26" s="7"/>
-      <c r="E26" s="7">
+      <c r="E26" s="21">
         <v>3</v>
       </c>
+      <c r="F26" s="24"/>
     </row>
     <row r="27" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="5">
@@ -929,9 +1027,10 @@
       <c r="B27" s="13"/>
       <c r="C27" s="13"/>
       <c r="D27" s="7"/>
-      <c r="E27" s="7">
+      <c r="E27" s="21">
         <v>1</v>
       </c>
+      <c r="F27" s="24"/>
     </row>
     <row r="28" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="5">
@@ -940,9 +1039,10 @@
       <c r="B28" s="12"/>
       <c r="C28" s="12"/>
       <c r="D28" s="7"/>
-      <c r="E28" s="7">
+      <c r="E28" s="21">
         <v>2</v>
       </c>
+      <c r="F28" s="24"/>
     </row>
     <row r="29" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="5">
@@ -955,9 +1055,10 @@
         <v>44178.997916666667</v>
       </c>
       <c r="D29" s="7"/>
-      <c r="E29" s="7">
+      <c r="E29" s="21">
         <v>2</v>
       </c>
+      <c r="F29" s="24"/>
     </row>
     <row r="30" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="5">
@@ -972,9 +1073,10 @@
       <c r="D30" s="7">
         <v>19</v>
       </c>
-      <c r="E30" s="7">
+      <c r="E30" s="21">
         <v>3</v>
       </c>
+      <c r="F30" s="24"/>
     </row>
     <row r="31" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="5">
@@ -989,9 +1091,10 @@
       <c r="D31" s="7">
         <v>11</v>
       </c>
-      <c r="E31" s="7">
+      <c r="E31" s="21">
         <v>3</v>
       </c>
+      <c r="F31" s="24"/>
     </row>
     <row r="32" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="5">
@@ -1006,11 +1109,12 @@
       <c r="D32" s="7">
         <v>10</v>
       </c>
-      <c r="E32" s="7">
+      <c r="E32" s="21">
         <v>3</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F32" s="24"/>
+    </row>
+    <row r="33" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="5">
         <v>44243</v>
       </c>
@@ -1023,11 +1127,12 @@
       <c r="D33" s="7">
         <v>7</v>
       </c>
-      <c r="E33" s="7">
+      <c r="E33" s="21">
         <v>3</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F33" s="24"/>
+    </row>
+    <row r="34" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="5">
         <v>44245</v>
       </c>
@@ -1040,11 +1145,12 @@
       <c r="D34" s="7">
         <v>6</v>
       </c>
-      <c r="E34" s="7">
+      <c r="E34" s="21">
         <v>3</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F34" s="24"/>
+    </row>
+    <row r="35" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="5">
         <v>44246</v>
       </c>
@@ -1057,11 +1163,12 @@
       <c r="D35" s="7">
         <v>14</v>
       </c>
-      <c r="E35" s="7">
+      <c r="E35" s="21">
         <v>1</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F35" s="24"/>
+    </row>
+    <row r="36" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="5">
         <v>44248</v>
       </c>
@@ -1074,11 +1181,14 @@
       <c r="D36" s="7">
         <v>25</v>
       </c>
-      <c r="E36" s="7">
+      <c r="E36" s="21">
         <v>1</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F36" s="24" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="5">
         <v>44249</v>
       </c>
@@ -1091,11 +1201,14 @@
       <c r="D37" s="7">
         <v>40</v>
       </c>
-      <c r="E37" s="7">
+      <c r="E37" s="21">
         <v>4</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F37" s="24" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="5">
         <v>44251</v>
       </c>
@@ -1108,11 +1221,12 @@
       <c r="D38" s="7">
         <v>10</v>
       </c>
-      <c r="E38" s="7">
+      <c r="E38" s="21">
         <v>4</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F38" s="24"/>
+    </row>
+    <row r="39" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="5">
         <v>44255</v>
       </c>
@@ -1125,11 +1239,12 @@
       <c r="D39" s="7">
         <v>16</v>
       </c>
-      <c r="E39" s="7">
+      <c r="E39" s="21">
         <v>1</v>
       </c>
-    </row>
-    <row r="40" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F39" s="24"/>
+    </row>
+    <row r="40" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="5">
         <v>44257</v>
       </c>
@@ -1142,11 +1257,12 @@
       <c r="D40" s="7">
         <v>15</v>
       </c>
-      <c r="E40" s="7">
+      <c r="E40" s="21">
         <v>1</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F40" s="24"/>
+    </row>
+    <row r="41" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="5">
         <v>44259</v>
       </c>
@@ -1159,11 +1275,14 @@
       <c r="D41" s="7">
         <v>22</v>
       </c>
-      <c r="E41" s="7">
+      <c r="E41" s="21">
         <v>1</v>
       </c>
-    </row>
-    <row r="42" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F41" s="24" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="5">
         <v>44262</v>
       </c>
@@ -1176,11 +1295,12 @@
       <c r="D42" s="7">
         <v>10</v>
       </c>
-      <c r="E42" s="7">
+      <c r="E42" s="21">
         <v>1</v>
       </c>
-    </row>
-    <row r="43" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F42" s="24"/>
+    </row>
+    <row r="43" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="5">
         <v>44265</v>
       </c>
@@ -1193,11 +1313,12 @@
       <c r="D43" s="7">
         <v>17</v>
       </c>
-      <c r="E43" s="7">
+      <c r="E43" s="21">
         <v>3</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F43" s="24"/>
+    </row>
+    <row r="44" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="5">
         <v>44267</v>
       </c>
@@ -1210,11 +1331,14 @@
       <c r="D44" s="7">
         <v>21</v>
       </c>
-      <c r="E44" s="7">
+      <c r="E44" s="21">
         <v>1</v>
       </c>
-    </row>
-    <row r="45" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F44" s="24" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="5">
         <v>44270</v>
       </c>
@@ -1225,11 +1349,12 @@
         <v>44270.122916666667</v>
       </c>
       <c r="D45" s="7"/>
-      <c r="E45" s="7">
+      <c r="E45" s="21">
         <v>3</v>
       </c>
-    </row>
-    <row r="46" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F45" s="24"/>
+    </row>
+    <row r="46" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="5">
         <v>44272</v>
       </c>
@@ -1240,11 +1365,12 @@
         <v>44272.268750000003</v>
       </c>
       <c r="D46" s="7"/>
-      <c r="E46" s="7">
+      <c r="E46" s="21">
         <v>4</v>
       </c>
-    </row>
-    <row r="47" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F46" s="24"/>
+    </row>
+    <row r="47" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="5">
         <v>44274</v>
       </c>
@@ -1257,11 +1383,12 @@
       <c r="D47" s="7">
         <v>9</v>
       </c>
-      <c r="E47" s="7">
+      <c r="E47" s="21">
         <v>3</v>
       </c>
-    </row>
-    <row r="48" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F47" s="24"/>
+    </row>
+    <row r="48" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="5">
         <v>44279</v>
       </c>
@@ -1272,11 +1399,12 @@
         <v>44279.372916666667</v>
       </c>
       <c r="D48" s="7"/>
-      <c r="E48" s="7">
+      <c r="E48" s="21">
         <v>3</v>
       </c>
-    </row>
-    <row r="49" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F48" s="24"/>
+    </row>
+    <row r="49" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="5">
         <v>44287</v>
       </c>
@@ -1287,11 +1415,12 @@
         <v>44287.654166666667</v>
       </c>
       <c r="D49" s="7"/>
-      <c r="E49" s="7">
+      <c r="E49" s="21">
         <v>4</v>
       </c>
-    </row>
-    <row r="50" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F49" s="24"/>
+    </row>
+    <row r="50" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="5">
         <v>44335</v>
       </c>
@@ -1302,11 +1431,12 @@
         <v>44335.227083333331</v>
       </c>
       <c r="D50" s="7"/>
-      <c r="E50" s="7">
+      <c r="E50" s="21">
         <v>2</v>
       </c>
-    </row>
-    <row r="51" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F50" s="24"/>
+    </row>
+    <row r="51" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="5">
         <v>44337</v>
       </c>
@@ -1317,11 +1447,12 @@
         <v>44337.143750000003</v>
       </c>
       <c r="D51" s="7"/>
-      <c r="E51" s="7">
+      <c r="E51" s="21">
         <v>2</v>
       </c>
-    </row>
-    <row r="52" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F51" s="24"/>
+    </row>
+    <row r="52" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="5">
         <v>44338</v>
       </c>
@@ -1332,11 +1463,12 @@
         <v>44338.977083333331</v>
       </c>
       <c r="D52" s="7"/>
-      <c r="E52" s="7">
+      <c r="E52" s="21">
         <v>2</v>
       </c>
-    </row>
-    <row r="53" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F52" s="24"/>
+    </row>
+    <row r="53" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="5">
         <v>44340</v>
       </c>
@@ -1349,11 +1481,12 @@
       <c r="D53" s="7">
         <v>12</v>
       </c>
-      <c r="E53" s="7">
+      <c r="E53" s="21">
         <v>2</v>
       </c>
-    </row>
-    <row r="54" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F53" s="24"/>
+    </row>
+    <row r="54" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="5">
         <v>44341</v>
       </c>
@@ -1364,11 +1497,12 @@
         <v>44341.872916666667</v>
       </c>
       <c r="D54" s="7"/>
-      <c r="E54" s="7">
+      <c r="E54" s="21">
         <v>3</v>
       </c>
-    </row>
-    <row r="55" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F54" s="24"/>
+    </row>
+    <row r="55" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="5">
         <v>44342</v>
       </c>
@@ -1379,11 +1513,12 @@
         <v>44342.55</v>
       </c>
       <c r="D55" s="7"/>
-      <c r="E55" s="7">
+      <c r="E55" s="21">
         <v>2</v>
       </c>
-    </row>
-    <row r="56" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F55" s="24"/>
+    </row>
+    <row r="56" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="5">
         <v>44346</v>
       </c>
@@ -1394,11 +1529,12 @@
         <v>44346.331250000003</v>
       </c>
       <c r="D56" s="7"/>
-      <c r="E56" s="7">
+      <c r="E56" s="21">
         <v>3</v>
       </c>
-    </row>
-    <row r="57" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F56" s="24"/>
+    </row>
+    <row r="57" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="5">
         <v>44349</v>
       </c>
@@ -1409,11 +1545,12 @@
         <v>44349.497916666667</v>
       </c>
       <c r="D57" s="7"/>
-      <c r="E57" s="7">
+      <c r="E57" s="21">
         <v>3</v>
       </c>
-    </row>
-    <row r="58" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F57" s="24"/>
+    </row>
+    <row r="58" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="5">
         <v>44351</v>
       </c>
@@ -1426,11 +1563,12 @@
       <c r="D58" s="7">
         <v>9</v>
       </c>
-      <c r="E58" s="7">
+      <c r="E58" s="21">
         <v>1</v>
       </c>
-    </row>
-    <row r="59" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F58" s="24"/>
+    </row>
+    <row r="59" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="5">
         <v>44359</v>
       </c>
@@ -1441,11 +1579,12 @@
         <v>44359.997916666667</v>
       </c>
       <c r="D59" s="7"/>
-      <c r="E59" s="7">
+      <c r="E59" s="21">
         <v>3</v>
       </c>
-    </row>
-    <row r="60" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F59" s="24"/>
+    </row>
+    <row r="60" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="5">
         <v>44361</v>
       </c>
@@ -1458,11 +1597,12 @@
       <c r="D60" s="7">
         <v>8</v>
       </c>
-      <c r="E60" s="7">
+      <c r="E60" s="21">
         <v>1</v>
       </c>
-    </row>
-    <row r="61" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F60" s="24"/>
+    </row>
+    <row r="61" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="5">
         <v>44363</v>
       </c>
@@ -1475,11 +1615,12 @@
       <c r="D61" s="7">
         <v>15</v>
       </c>
-      <c r="E61" s="7">
+      <c r="E61" s="21">
         <v>1</v>
       </c>
-    </row>
-    <row r="62" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F61" s="24"/>
+    </row>
+    <row r="62" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="5">
         <v>44364</v>
       </c>
@@ -1490,11 +1631,12 @@
         <v>44365.164583333331</v>
       </c>
       <c r="D62" s="7"/>
-      <c r="E62" s="7">
+      <c r="E62" s="21">
         <v>3</v>
       </c>
-    </row>
-    <row r="63" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F62" s="24"/>
+    </row>
+    <row r="63" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="5">
         <v>44366</v>
       </c>
@@ -1505,11 +1647,12 @@
         <v>44366.966666666667</v>
       </c>
       <c r="D63" s="7"/>
-      <c r="E63" s="7">
+      <c r="E63" s="21">
         <v>4</v>
       </c>
-    </row>
-    <row r="64" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F63" s="24"/>
+    </row>
+    <row r="64" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="5">
         <v>44367</v>
       </c>
@@ -1522,9 +1665,10 @@
       <c r="D64" s="7">
         <v>10</v>
       </c>
-      <c r="E64" s="7">
+      <c r="E64" s="21">
         <v>3</v>
       </c>
+      <c r="F64" s="24"/>
     </row>
     <row r="65" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="5">
@@ -1537,9 +1681,10 @@
         <v>44369.372916666667</v>
       </c>
       <c r="D65" s="7"/>
-      <c r="E65" s="7">
+      <c r="E65" s="21">
         <v>3</v>
       </c>
+      <c r="F65" s="24"/>
     </row>
     <row r="66" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="5">
@@ -1554,9 +1699,10 @@
       <c r="D66" s="7">
         <v>14</v>
       </c>
-      <c r="E66" s="7">
+      <c r="E66" s="21">
         <v>1</v>
       </c>
+      <c r="F66" s="24"/>
     </row>
     <row r="67" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="5">
@@ -1569,9 +1715,10 @@
         <v>44370.904166666667</v>
       </c>
       <c r="D67" s="7"/>
-      <c r="E67" s="7">
+      <c r="E67" s="21">
         <v>3</v>
       </c>
+      <c r="F67" s="24"/>
     </row>
     <row r="68" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="5">
@@ -1586,9 +1733,10 @@
       <c r="D68" s="7">
         <v>8</v>
       </c>
-      <c r="E68" s="7">
+      <c r="E68" s="21">
         <v>3</v>
       </c>
+      <c r="F68" s="24"/>
     </row>
     <row r="69" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="5">
@@ -1603,9 +1751,10 @@
       <c r="D69" s="7">
         <v>6</v>
       </c>
-      <c r="E69" s="7">
+      <c r="E69" s="21">
         <v>1</v>
       </c>
+      <c r="F69" s="24"/>
     </row>
     <row r="70" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="5">
@@ -1618,9 +1767,10 @@
         <v>44372.997916666667</v>
       </c>
       <c r="D70" s="7"/>
-      <c r="E70" s="7">
+      <c r="E70" s="21">
         <v>1</v>
       </c>
+      <c r="F70" s="24"/>
     </row>
     <row r="71" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="5">
@@ -1633,9 +1783,10 @@
         <v>44373.831250000003</v>
       </c>
       <c r="D71" s="7"/>
-      <c r="E71" s="7">
+      <c r="E71" s="21">
         <v>3</v>
       </c>
+      <c r="F71" s="24"/>
     </row>
     <row r="72" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="5">
@@ -1648,9 +1799,10 @@
         <v>44374.456250000003</v>
       </c>
       <c r="D72" s="7"/>
-      <c r="E72" s="7">
+      <c r="E72" s="21">
         <v>3</v>
       </c>
+      <c r="F72" s="24"/>
     </row>
     <row r="73" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" s="5">
@@ -1665,9 +1817,10 @@
       <c r="D73" s="7">
         <v>15</v>
       </c>
-      <c r="E73" s="7">
+      <c r="E73" s="21">
         <v>3</v>
       </c>
+      <c r="F73" s="24"/>
     </row>
     <row r="74" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="5">
@@ -1680,9 +1833,10 @@
         <v>44379.060416666667</v>
       </c>
       <c r="D74" s="7"/>
-      <c r="E74" s="7">
+      <c r="E74" s="21">
         <v>3</v>
       </c>
+      <c r="F74" s="24"/>
     </row>
     <row r="75" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="5">
@@ -1695,9 +1849,10 @@
         <v>44381.758333333331</v>
       </c>
       <c r="D75" s="7"/>
-      <c r="E75" s="7">
+      <c r="E75" s="21">
         <v>3</v>
       </c>
+      <c r="F75" s="24"/>
       <c r="J75" s="11"/>
     </row>
     <row r="76" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -1713,9 +1868,10 @@
       <c r="D76" s="7">
         <v>17</v>
       </c>
-      <c r="E76" s="7">
+      <c r="E76" s="21">
         <v>1</v>
       </c>
+      <c r="F76" s="24"/>
     </row>
     <row r="77" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A77" s="5">
@@ -1730,9 +1886,10 @@
       <c r="D77" s="7">
         <v>12</v>
       </c>
-      <c r="E77" s="7">
+      <c r="E77" s="21">
         <v>1</v>
       </c>
+      <c r="F77" s="24"/>
     </row>
     <row r="78" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" s="5">
@@ -1745,9 +1902,10 @@
         <v>44391.581250000003</v>
       </c>
       <c r="D78" s="7"/>
-      <c r="E78" s="7">
+      <c r="E78" s="21">
         <v>3</v>
       </c>
+      <c r="F78" s="24"/>
     </row>
     <row r="79" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" s="5">
@@ -1762,9 +1920,10 @@
       <c r="D79" s="7">
         <v>12</v>
       </c>
-      <c r="E79" s="7">
+      <c r="E79" s="21">
         <v>3</v>
       </c>
+      <c r="F79" s="24"/>
     </row>
     <row r="80" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A80" s="5">
@@ -1779,9 +1938,10 @@
       <c r="D80" s="7">
         <v>23</v>
       </c>
-      <c r="E80" s="7">
+      <c r="E80" s="21">
         <v>1</v>
       </c>
+      <c r="F80" s="24"/>
     </row>
     <row r="81" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A81" s="5">
@@ -1796,9 +1956,10 @@
       <c r="D81" s="7">
         <v>20</v>
       </c>
-      <c r="E81" s="7">
+      <c r="E81" s="21">
         <v>1</v>
       </c>
+      <c r="F81" s="24"/>
     </row>
     <row r="82" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="5">
@@ -1813,9 +1974,10 @@
       <c r="D82" s="7">
         <v>12</v>
       </c>
-      <c r="E82" s="7">
+      <c r="E82" s="21">
         <v>1</v>
       </c>
+      <c r="F82" s="24"/>
     </row>
     <row r="83" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A83" s="5">
@@ -1830,9 +1992,10 @@
       <c r="D83" s="7">
         <v>11</v>
       </c>
-      <c r="E83" s="7">
+      <c r="E83" s="21">
         <v>3</v>
       </c>
+      <c r="F83" s="24"/>
     </row>
     <row r="84" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A84" s="5">
@@ -1847,9 +2010,10 @@
       <c r="D84" s="7">
         <v>11</v>
       </c>
-      <c r="E84" s="7">
+      <c r="E84" s="21">
         <v>3</v>
       </c>
+      <c r="F84" s="24"/>
     </row>
     <row r="85" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A85" s="5">
@@ -1864,9 +2028,10 @@
       <c r="D85" s="7">
         <v>13</v>
       </c>
-      <c r="E85" s="7">
+      <c r="E85" s="21">
         <v>1</v>
       </c>
+      <c r="F85" s="24"/>
     </row>
     <row r="86" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A86" s="5">
@@ -1881,9 +2046,10 @@
       <c r="D86" s="7">
         <v>17</v>
       </c>
-      <c r="E86" s="7">
+      <c r="E86" s="21">
         <v>1</v>
       </c>
+      <c r="F86" s="24"/>
     </row>
     <row r="87" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A87" s="5">
@@ -1898,9 +2064,10 @@
       <c r="D87" s="7">
         <v>48</v>
       </c>
-      <c r="E87" s="7">
+      <c r="E87" s="21">
         <v>3</v>
       </c>
+      <c r="F87" s="24"/>
     </row>
     <row r="88" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A88" s="5">
@@ -1915,9 +2082,10 @@
       <c r="D88" s="7">
         <v>25</v>
       </c>
-      <c r="E88" s="7">
+      <c r="E88" s="21">
         <v>4</v>
       </c>
+      <c r="F88" s="24"/>
     </row>
     <row r="89" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A89" s="5">
@@ -1932,9 +2100,10 @@
       <c r="D89" s="7">
         <v>30</v>
       </c>
-      <c r="E89" s="7">
+      <c r="E89" s="21">
         <v>1</v>
       </c>
+      <c r="F89" s="24"/>
     </row>
     <row r="90" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A90" s="5">
@@ -1949,9 +2118,10 @@
       <c r="D90" s="7">
         <v>12</v>
       </c>
-      <c r="E90" s="7">
+      <c r="E90" s="21">
         <v>3</v>
       </c>
+      <c r="F90" s="24"/>
     </row>
     <row r="91" spans="1:26" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A91" s="5">
@@ -1966,9 +2136,10 @@
       <c r="D91" s="7">
         <v>14</v>
       </c>
-      <c r="E91" s="7">
+      <c r="E91" s="21">
         <v>4</v>
       </c>
+      <c r="F91" s="24"/>
     </row>
     <row r="92" spans="1:26" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A92" s="5">
@@ -1981,13 +2152,13 @@
         <v>45519.497916666667</v>
       </c>
       <c r="D92" s="7"/>
-      <c r="E92" s="7">
+      <c r="E92" s="21">
         <v>4</v>
       </c>
-      <c r="F92" s="15"/>
-      <c r="G92" s="15"/>
+      <c r="F92" s="24"/>
+      <c r="G92" s="22"/>
       <c r="H92" s="15"/>
-      <c r="I92" s="19"/>
+      <c r="I92" s="18"/>
       <c r="J92" s="15"/>
       <c r="K92" s="15"/>
       <c r="L92" s="15"/>
@@ -2009,7 +2180,7 @@
     <row r="93" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A93" s="9"/>
       <c r="D93" s="8"/>
-      <c r="E93" s="18"/>
+      <c r="E93" s="17"/>
     </row>
     <row r="94" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A94" s="9"/>

</xml_diff>